<commit_message>
Add special ability as well
</commit_message>
<xml_diff>
--- a/Element/Element.xlsx
+++ b/Element/Element.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SteamLibrary\steamapps\common\Elin\Package\Mod_PandaRodRechargeMod\Element\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B45A823-DCE6-4754-BC11-96119D12782F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93C3E2D-F1E5-482E-BCF3-E647B7E7BC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Element" sheetId="4" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="80">
   <si>
     <t>id</t>
   </si>
@@ -256,6 +256,42 @@
   </si>
   <si>
     <t>None</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>actRecharge</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>ABILITY</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>spRecharge</t>
+  </si>
+  <si>
+    <t>addEleOnLoad</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>act</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="游ゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Recharge</t>
+    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -263,7 +299,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="游ゴシック"/>
@@ -335,6 +371,12 @@
       <family val="2"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -376,7 +418,7 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -415,6 +457,7 @@
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Excel Built-in Normal" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
@@ -1077,35 +1120,83 @@
       <c r="AT4" s="2"/>
       <c r="AU4" s="2"/>
     </row>
-    <row r="5" spans="1:57">
-      <c r="A5" s="7"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
+    <row r="5" spans="1:57" ht="17.25" thickBot="1">
+      <c r="A5" s="7">
+        <v>12345678</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="11">
+        <v>5</v>
+      </c>
+      <c r="K5" s="11">
+        <v>100</v>
+      </c>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="11">
+        <v>100</v>
+      </c>
+      <c r="P5" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="13">
+        <v>1950</v>
+      </c>
+      <c r="R5" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="S5" s="9"/>
       <c r="T5" s="5"/>
-      <c r="U5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
-      <c r="AB5" s="2"/>
-      <c r="AD5" s="5"/>
-      <c r="AE5" s="5"/>
-      <c r="AF5" s="2"/>
-      <c r="AG5" s="5"/>
-      <c r="AH5" s="2"/>
-      <c r="AK5" s="5"/>
-      <c r="AR5" s="4"/>
-      <c r="AS5" s="2"/>
+      <c r="U5" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="W5" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="X5" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y5" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z5" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC5" s="9"/>
+      <c r="AD5" s="10"/>
+      <c r="AE5" s="9"/>
+      <c r="AF5" s="9"/>
+      <c r="AG5" s="9"/>
+      <c r="AH5" s="9"/>
+      <c r="AI5" s="9"/>
+      <c r="AJ5" s="9"/>
+      <c r="AK5" s="9"/>
+      <c r="AR5" t="s">
+        <v>62</v>
+      </c>
+      <c r="AS5" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="AT5" s="2"/>
       <c r="AU5" s="2"/>
     </row>

</xml_diff>

<commit_message>
Update to actually allow spawning scrolls of Recharge
</commit_message>
<xml_diff>
--- a/Element/Element.xlsx
+++ b/Element/Element.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SteamLibrary\steamapps\common\Elin\Package\Mod_PandaRodRechargeMod\Element\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93C3E2D-F1E5-482E-BCF3-E647B7E7BC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5BC0E0-AE79-49E5-8AAC-A8FDD710EA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Element" sheetId="4" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="78">
   <si>
     <t>id</t>
   </si>
@@ -238,10 +238,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>1</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>SPELL</t>
   </si>
   <si>
@@ -249,10 +245,6 @@
   </si>
   <si>
     <t>util</t>
-  </si>
-  <si>
-    <t>B S</t>
-    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>None</t>
@@ -268,10 +260,6 @@
   </si>
   <si>
     <t>spRecharge</t>
-  </si>
-  <si>
-    <t>addEleOnLoad</t>
-    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -294,12 +282,16 @@
     </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
+  <si>
+    <t>B SR</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="游ゴシック"/>
@@ -366,13 +358,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="游ゴシック"/>
-      <family val="2"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <name val="游ゴシック"/>
       <family val="2"/>
       <charset val="136"/>
@@ -418,7 +403,7 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -451,13 +436,7 @@
     <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Excel Built-in Normal" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
@@ -1066,18 +1045,20 @@
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="11">
+      <c r="N4" s="9">
+        <v>1</v>
+      </c>
+      <c r="O4" s="9">
+        <v>5</v>
+      </c>
+      <c r="P4" s="9">
         <v>100</v>
       </c>
-      <c r="P4" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="13">
-        <v>1950</v>
-      </c>
-      <c r="R4" s="11" t="s">
-        <v>69</v>
+      <c r="Q4" s="9">
+        <v>320</v>
+      </c>
+      <c r="R4" s="9">
+        <v>12</v>
       </c>
       <c r="S4" s="9"/>
       <c r="T4" s="5"/>
@@ -1085,23 +1066,23 @@
         <v>64</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="W4" t="s">
         <v>61</v>
       </c>
       <c r="X4" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y4" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="Y4" s="9" t="s">
+      <c r="Z4" s="9" t="s">
         <v>71</v>
-      </c>
-      <c r="Z4" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="AB4" s="2"/>
       <c r="AC4" s="9" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="AD4" s="10"/>
       <c r="AE4" s="9"/>
@@ -1125,7 +1106,7 @@
         <v>12345678</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>59</v>
@@ -1146,18 +1127,20 @@
       </c>
       <c r="L5" s="9"/>
       <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="11">
+      <c r="N5" s="9">
+        <v>1</v>
+      </c>
+      <c r="O5" s="9">
+        <v>5</v>
+      </c>
+      <c r="P5" s="9">
         <v>100</v>
       </c>
-      <c r="P5" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="13">
-        <v>1950</v>
-      </c>
-      <c r="R5" s="11" t="s">
-        <v>69</v>
+      <c r="Q5" s="9">
+        <v>320</v>
+      </c>
+      <c r="R5" s="9">
+        <v>12</v>
       </c>
       <c r="S5" s="9"/>
       <c r="T5" s="5"/>
@@ -1165,23 +1148,21 @@
         <v>64</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="W5" s="14" t="s">
-        <v>79</v>
+        <v>75</v>
+      </c>
+      <c r="W5" s="12" t="s">
+        <v>76</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Y5" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="Z5" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="Z5" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="AB5" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="AB5" s="2"/>
       <c r="AC5" s="9"/>
       <c r="AD5" s="10"/>
       <c r="AE5" s="9"/>

</xml_diff>